<commit_message>
Additional  file from reallocation of vehicle types
</commit_message>
<xml_diff>
--- a/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
+++ b/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\trans\SoCDTtiNTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea-ci\InputData\trans\SoCDTtiNTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EF0957-B562-4E54-8945-54421D16958F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1A8964-98DB-4AA4-BED4-2CA2BD5126D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43725" yWindow="3000" windowWidth="20145" windowHeight="11235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38505" yWindow="-4650" windowWidth="19410" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,7 @@
     <sheet name="SoCDTtiNTY-psgr" sheetId="2" r:id="rId3"/>
     <sheet name="SoCDTtiNTY-frgt" sheetId="4" r:id="rId4"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId5"/>
-  </externalReferences>
-  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -137,7 +134,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,6 +155,13 @@
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="3"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -214,62 +218,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="About"/>
-      <sheetName val="NTS 1-20"/>
-      <sheetName val="Data"/>
-      <sheetName val="SK calcs"/>
-      <sheetName val="AVL"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2">
-        <row r="16">
-          <cell r="A16">
-            <v>24</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="C22">
-            <v>34</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="C28">
-            <v>33</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="A48">
-            <v>17.22332068760786</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3">
-        <row r="36">
-          <cell r="J36">
-            <v>15.4</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="J37">
-            <v>16.8</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="4" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -560,14 +508,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -575,52 +523,53 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="B5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -628,9 +577,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DE974D0-35AB-448C-ABAC-291E7575B7A2}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="43.5">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -641,90 +590,78 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="8">
-        <f>'[1]SK calcs'!J36</f>
-        <v>15.4</v>
+        <v>15.6</v>
       </c>
       <c r="C2" s="8">
-        <f t="shared" ref="C2:C7" si="0">B2</f>
-        <v>15.4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>17.75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="8">
-        <f>'[1]SK calcs'!J37</f>
-        <v>16.8</v>
+        <v>15.5</v>
       </c>
       <c r="C3" s="8">
-        <f t="shared" si="0"/>
-        <v>16.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>17.75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="6">
-        <f>ROUND([1]Data!A16,0)</f>
         <v>24</v>
       </c>
       <c r="C4" s="6">
-        <f t="shared" si="0"/>
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
       <c r="B5">
-        <f>ROUND([1]Data!C22,0)</f>
         <v>34</v>
       </c>
       <c r="C5">
-        <f t="shared" si="0"/>
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
       <c r="B6">
-        <f>ROUND([1]Data!C28,0)</f>
         <v>33</v>
       </c>
       <c r="C6">
-        <f t="shared" si="0"/>
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
       <c r="B7">
-        <f>ROUND([1]Data!A48,0)</f>
         <v>17</v>
       </c>
       <c r="C7">
-        <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="43.5">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -735,85 +672,86 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="7">
         <f>1/B2</f>
-        <v>6.4935064935064929E-2</v>
+        <v>6.4102564102564111E-2</v>
       </c>
       <c r="C11" s="7">
         <f>1/C2</f>
-        <v>6.4935064935064929E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>5.6338028169014086E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="7">
-        <f t="shared" ref="B12:C16" si="1">1/B3</f>
-        <v>5.9523809523809521E-2</v>
+        <f t="shared" ref="B12:C16" si="0">1/B3</f>
+        <v>6.4516129032258063E-2</v>
       </c>
       <c r="C12" s="7">
-        <f t="shared" si="1"/>
-        <v>5.9523809523809521E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>5.6338028169014086E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="C13" s="7">
-        <f t="shared" si="1"/>
-        <v>4.1666666666666664E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666664E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.9411764705882353E-2</v>
       </c>
       <c r="C14" s="7">
-        <f t="shared" si="1"/>
-        <v>2.9411764705882353E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>2.9411764705882353E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3.0303030303030304E-2</v>
       </c>
       <c r="C15" s="7">
-        <f t="shared" si="1"/>
-        <v>3.0303030303030304E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>3.0303030303030304E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5.8823529411764705E-2</v>
       </c>
       <c r="C16" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5.8823529411764705E-2</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -824,13 +762,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.109375" customWidth="1"/>
-    <col min="2" max="8" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="19.08984375" customWidth="1"/>
+    <col min="2" max="8" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="29">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -856,73 +794,73 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2">
         <f>AVL!$B$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>6.4102564102564111E-2</v>
       </c>
       <c r="C2">
         <f>AVL!$B$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>6.4102564102564111E-2</v>
       </c>
       <c r="D2">
         <f>AVL!$B$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>6.4102564102564111E-2</v>
       </c>
       <c r="E2">
         <f>AVL!$B$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>6.4102564102564111E-2</v>
       </c>
       <c r="F2">
         <f>AVL!$B$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>6.4102564102564111E-2</v>
       </c>
       <c r="G2">
         <f>AVL!$B$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>6.4102564102564111E-2</v>
       </c>
       <c r="H2">
         <f>AVL!$B$11</f>
-        <v>6.4935064935064929E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>6.4102564102564111E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3">
         <f>AVL!$B$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>6.4516129032258063E-2</v>
       </c>
       <c r="C3">
         <f>AVL!$B$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>6.4516129032258063E-2</v>
       </c>
       <c r="D3">
         <f>AVL!$B$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>6.4516129032258063E-2</v>
       </c>
       <c r="E3">
         <f>AVL!$B$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>6.4516129032258063E-2</v>
       </c>
       <c r="F3">
         <f>AVL!$B$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>6.4516129032258063E-2</v>
       </c>
       <c r="G3">
         <f>AVL!$B$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>6.4516129032258063E-2</v>
       </c>
       <c r="H3">
         <f>AVL!$B$12</f>
-        <v>5.9523809523809521E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>6.4516129032258063E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -955,7 +893,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -988,7 +926,7 @@
         <v>2.9411764705882353E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1021,7 +959,7 @@
         <v>3.0303030303030304E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -1055,6 +993,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1065,13 +1004,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.109375" customWidth="1"/>
-    <col min="2" max="8" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="19.08984375" customWidth="1"/>
+    <col min="2" max="8" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="29">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -1097,73 +1036,73 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2">
         <f>AVL!$C$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="C2">
         <f>AVL!$C$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="D2">
         <f>AVL!$C$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="E2">
         <f>AVL!$C$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="F2">
         <f>AVL!$C$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="G2">
         <f>AVL!$C$11</f>
-        <v>6.4935064935064929E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="H2">
         <f>AVL!$C$11</f>
-        <v>6.4935064935064929E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>5.6338028169014086E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3">
         <f>AVL!$C$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="C3">
         <f>AVL!$C$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="D3">
         <f>AVL!$C$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="E3">
         <f>AVL!$C$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="F3">
         <f>AVL!$C$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="G3">
         <f>AVL!$C$12</f>
-        <v>5.9523809523809521E-2</v>
+        <v>5.6338028169014086E-2</v>
       </c>
       <c r="H3">
         <f>AVL!$C$12</f>
-        <v>5.9523809523809521E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>5.6338028169014086E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1196,7 +1135,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1229,7 +1168,7 @@
         <v>2.9411764705882353E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1262,7 +1201,7 @@
         <v>3.0303030303030304E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -1296,26 +1235,12 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -1459,24 +1384,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A502D4-C09A-449A-A258-EE541B816382}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{441C2D10-A603-4499-828F-5FADDAF9DE77}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149AAAE-ABCC-460E-97F6-A6D332D4802A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1492,4 +1415,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A502D4-C09A-449A-A258-EE541B816382}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{441C2D10-A603-4499-828F-5FADDAF9DE77}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Transportation sector calibration updates
</commit_message>
<xml_diff>
--- a/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
+++ b/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\SK\eps-southkorea\InputData\trans\SoCDTtiNTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\trans\SoCDTtiNTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E6DABE7-05FE-4BD2-AB7D-D541D2E0685D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E18B893-E8CA-4EA1-96E1-8AA111939D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25260" yWindow="1515" windowWidth="24345" windowHeight="13980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -799,32 +799,25 @@
         <v>12</v>
       </c>
       <c r="B2">
-        <f>AVL!$B$11</f>
-        <v>7.6923076923076927E-2</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="C2">
-        <f>AVL!$B$11</f>
-        <v>7.6923076923076927E-2</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="D2">
-        <f>AVL!$B$11</f>
-        <v>7.6923076923076927E-2</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="E2">
-        <f>AVL!$B$11</f>
-        <v>7.6923076923076927E-2</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="F2">
-        <f>AVL!$B$11</f>
-        <v>7.6923076923076927E-2</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="G2">
-        <f>AVL!$B$11</f>
-        <v>7.6923076923076927E-2</v>
+        <v>6.7000000000000004E-2</v>
       </c>
       <c r="H2">
-        <f>AVL!$B$11</f>
-        <v>7.6923076923076927E-2</v>
+        <v>6.7000000000000004E-2</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1241,9 +1234,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1391,19 +1387,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A502D4-C09A-449A-A258-EE541B816382}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{441C2D10-A603-4499-828F-5FADDAF9DE77}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1427,9 +1419,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{441C2D10-A603-4499-828F-5FADDAF9DE77}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A502D4-C09A-449A-A258-EE541B816382}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>